<commit_message>
fix: nuevos datos y crear ExcelSoli
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/excel/ACTA DE VISITA.xlsx
+++ b/backend/src/main/resources/templates/excel/ACTA DE VISITA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d3fcf720eca7cd5b/Documentos/DEFENSORIA/TURNO/NOVIEMBRE/LUIS ALBERTO ESALA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP VICTUS\IdeaProjects\create_actas\backend\src\main\resources\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D6CA2DB-7DEF-483F-B776-CB3BFE22EEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15976FBA-F768-40E0-9E7A-C5E98A2083A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -144,9 +144,6 @@
     <t>BOLIVAR</t>
   </si>
   <si>
-    <t>SI: X</t>
-  </si>
-  <si>
     <t>INDICIADO</t>
   </si>
   <si>
@@ -191,6 +188,9 @@
   </si>
   <si>
     <t>13 001 60 01129 2025 08665.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SI: </t>
   </si>
 </sst>
 </file>
@@ -499,15 +499,51 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -564,42 +600,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -961,21 +961,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.26953125" customWidth="1"/>
-    <col min="2" max="2" width="1.54296875" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" customWidth="1"/>
-    <col min="4" max="4" width="14.7265625" customWidth="1"/>
-    <col min="5" max="6" width="12.7265625" customWidth="1"/>
-    <col min="7" max="8" width="14.7265625" customWidth="1"/>
-    <col min="9" max="9" width="10.1796875" customWidth="1"/>
-    <col min="10" max="11" width="8.7265625" customWidth="1"/>
-    <col min="12" max="12" width="7.7265625" customWidth="1"/>
-    <col min="13" max="13" width="4.7265625" customWidth="1"/>
+    <col min="1" max="1" width="1.21875" customWidth="1"/>
+    <col min="2" max="2" width="1.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" customWidth="1"/>
+    <col min="5" max="6" width="12.77734375" customWidth="1"/>
+    <col min="7" max="8" width="14.77734375" customWidth="1"/>
+    <col min="9" max="9" width="10.21875" customWidth="1"/>
+    <col min="10" max="11" width="8.77734375" customWidth="1"/>
+    <col min="12" max="12" width="7.77734375" customWidth="1"/>
+    <col min="13" max="13" width="4.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="6.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="6.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12"/>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -990,64 +990,64 @@
       <c r="L1" s="12"/>
       <c r="M1" s="12"/>
     </row>
-    <row r="2" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="36" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="30" t="s">
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="32"/>
-    </row>
-    <row r="3" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="44"/>
+    </row>
+    <row r="3" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="12"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="39" t="s">
+      <c r="B3" s="38"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="30" t="s">
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="32"/>
-    </row>
-    <row r="4" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="44"/>
+    </row>
+    <row r="4" spans="1:13" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="12"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="33" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="K4" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="34"/>
-      <c r="M4" s="35"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="L4" s="46"/>
+      <c r="M4" s="47"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="12"/>
       <c r="B5" s="1"/>
       <c r="C5" s="2"/>
@@ -1062,26 +1062,26 @@
       <c r="L5" s="2"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="12"/>
       <c r="B6" s="4"/>
       <c r="C6" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="6"/>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
       <c r="M6" s="5"/>
     </row>
-    <row r="7" spans="1:13" ht="7.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="12"/>
       <c r="B7" s="4"/>
       <c r="C7" s="7"/>
@@ -1096,45 +1096,45 @@
       <c r="L7" s="6"/>
       <c r="M7" s="5"/>
     </row>
-    <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12"/>
       <c r="B8" s="4"/>
       <c r="C8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
+      <c r="E8" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
       <c r="M8" s="5"/>
     </row>
-    <row r="9" spans="1:13" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:13" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="12"/>
       <c r="B9" s="4"/>
       <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="6"/>
-      <c r="E9" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
+      <c r="E9" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
       <c r="M9" s="5"/>
     </row>
-    <row r="10" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="4"/>
       <c r="C10" s="7"/>
@@ -1149,26 +1149,26 @@
       <c r="L10" s="6"/>
       <c r="M10" s="5"/>
     </row>
-    <row r="11" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="48"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
       <c r="M11" s="5"/>
     </row>
-    <row r="12" spans="1:13" ht="7.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="4"/>
       <c r="C12" s="6"/>
@@ -1183,26 +1183,26 @@
       <c r="L12" s="6"/>
       <c r="M12" s="5"/>
     </row>
-    <row r="13" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="12"/>
       <c r="B13" s="4"/>
       <c r="C13" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="6"/>
-      <c r="E13" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
+      <c r="E13" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="26"/>
       <c r="M13" s="5"/>
     </row>
-    <row r="14" spans="1:13" ht="7.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="4"/>
       <c r="C14" s="6"/>
@@ -1217,26 +1217,26 @@
       <c r="L14" s="6"/>
       <c r="M14" s="5"/>
     </row>
-    <row r="15" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="12"/>
       <c r="B15" s="4"/>
       <c r="C15" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D15" s="6"/>
-      <c r="E15" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
+      <c r="E15" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
       <c r="M15" s="5"/>
     </row>
-    <row r="16" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="12"/>
       <c r="B16" s="4"/>
       <c r="C16" s="6"/>
@@ -1251,26 +1251,26 @@
       <c r="L16" s="6"/>
       <c r="M16" s="5"/>
     </row>
-    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="12"/>
       <c r="B17" s="4"/>
       <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="6"/>
-      <c r="E17" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
+      <c r="E17" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
       <c r="M17" s="5"/>
     </row>
-    <row r="18" spans="1:13" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:13" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="12"/>
       <c r="B18" s="4"/>
       <c r="C18" s="6"/>
@@ -1285,7 +1285,7 @@
       <c r="L18" s="17"/>
       <c r="M18" s="5"/>
     </row>
-    <row r="19" spans="1:13" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:13" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="12"/>
       <c r="B19" s="4"/>
       <c r="C19" s="6" t="s">
@@ -1294,38 +1294,38 @@
       <c r="D19" s="15"/>
       <c r="E19" s="14"/>
       <c r="F19" s="16" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="G19" s="15"/>
       <c r="H19" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="I19" s="52"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
+        <v>31</v>
+      </c>
+      <c r="I19" s="31"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
       <c r="M19" s="5"/>
     </row>
-    <row r="20" spans="1:13" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:13" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="12"/>
       <c r="B20" s="4"/>
       <c r="C20" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D20" s="6"/>
-      <c r="E20" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
+      <c r="E20" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
       <c r="M20" s="5"/>
     </row>
-    <row r="21" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="12"/>
       <c r="B21" s="4"/>
       <c r="C21" s="6"/>
@@ -1340,7 +1340,7 @@
       <c r="L21" s="17"/>
       <c r="M21" s="5"/>
     </row>
-    <row r="22" spans="1:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12"/>
       <c r="B22" s="4"/>
       <c r="C22" s="6"/>
@@ -1355,28 +1355,28 @@
       <c r="L22" s="6"/>
       <c r="M22" s="5"/>
     </row>
-    <row r="23" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="12"/>
       <c r="B23" s="4"/>
       <c r="C23" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="6"/>
-      <c r="E23" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="51" t="s">
+      <c r="E23" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="I23" s="51"/>
+      <c r="I23" s="30"/>
       <c r="J23" s="21"/>
       <c r="K23" s="21"/>
       <c r="L23" s="21"/>
       <c r="M23" s="5"/>
     </row>
-    <row r="24" spans="1:13" ht="6.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="12"/>
       <c r="B24" s="4"/>
       <c r="C24" s="6"/>
@@ -1391,26 +1391,26 @@
       <c r="L24" s="13"/>
       <c r="M24" s="5"/>
     </row>
-    <row r="25" spans="1:13" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:13" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="12"/>
       <c r="B25" s="4"/>
       <c r="C25" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
+      <c r="E25" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
       <c r="M25" s="5"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="12"/>
       <c r="B26" s="4"/>
       <c r="C26" s="6"/>
@@ -1425,26 +1425,26 @@
       <c r="L26" s="6"/>
       <c r="M26" s="5"/>
     </row>
-    <row r="27" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="12"/>
       <c r="B27" s="4"/>
       <c r="C27" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="6"/>
-      <c r="E27" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
+      <c r="E27" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
       <c r="M27" s="5"/>
     </row>
-    <row r="28" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="12"/>
       <c r="B28" s="4"/>
       <c r="C28" s="9"/>
@@ -1459,26 +1459,26 @@
       <c r="L28" s="7"/>
       <c r="M28" s="5"/>
     </row>
-    <row r="29" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="12"/>
       <c r="B29" s="4"/>
-      <c r="C29" s="51" t="s">
+      <c r="C29" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="D29" s="51"/>
-      <c r="E29" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" s="49"/>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="49"/>
-      <c r="J29" s="49"/>
-      <c r="K29" s="49"/>
-      <c r="L29" s="49"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
       <c r="M29" s="5"/>
     </row>
-    <row r="30" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="12"/>
       <c r="B30" s="4"/>
       <c r="C30" s="7"/>
@@ -1493,11 +1493,11 @@
       <c r="L30" s="7"/>
       <c r="M30" s="5"/>
     </row>
-    <row r="31" spans="1:13" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:13" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="12"/>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
@@ -1510,7 +1510,7 @@
       <c r="L31" s="8"/>
       <c r="M31" s="5"/>
     </row>
-    <row r="32" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="12"/>
       <c r="B32" s="4"/>
       <c r="C32" s="7"/>
@@ -1525,11 +1525,11 @@
       <c r="L32" s="7"/>
       <c r="M32" s="5"/>
     </row>
-    <row r="33" spans="1:13" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:13" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="12"/>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
@@ -1542,7 +1542,7 @@
       <c r="L33" s="8"/>
       <c r="M33" s="5"/>
     </row>
-    <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12"/>
       <c r="B34" s="4"/>
       <c r="C34" s="7"/>
@@ -1557,11 +1557,11 @@
       <c r="L34" s="7"/>
       <c r="M34" s="5"/>
     </row>
-    <row r="35" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="12"/>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
@@ -1574,7 +1574,7 @@
       <c r="L35" s="8"/>
       <c r="M35" s="5"/>
     </row>
-    <row r="36" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="12"/>
       <c r="B36" s="4"/>
       <c r="C36" s="7"/>
@@ -1589,7 +1589,7 @@
       <c r="L36" s="7"/>
       <c r="M36" s="5"/>
     </row>
-    <row r="37" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="12"/>
       <c r="B37" s="4"/>
       <c r="C37" s="8"/>
@@ -1604,7 +1604,7 @@
       <c r="L37" s="8"/>
       <c r="M37" s="5"/>
     </row>
-    <row r="38" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="12"/>
       <c r="B38" s="4"/>
       <c r="C38" s="7"/>
@@ -1619,7 +1619,7 @@
       <c r="L38" s="7"/>
       <c r="M38" s="5"/>
     </row>
-    <row r="39" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="12"/>
       <c r="B39" s="4"/>
       <c r="C39" s="8"/>
@@ -1634,7 +1634,7 @@
       <c r="L39" s="8"/>
       <c r="M39" s="5"/>
     </row>
-    <row r="40" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="12"/>
       <c r="B40" s="4"/>
       <c r="C40" s="7"/>
@@ -1649,7 +1649,7 @@
       <c r="L40" s="7"/>
       <c r="M40" s="5"/>
     </row>
-    <row r="41" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="12"/>
       <c r="B41" s="4"/>
       <c r="C41" s="8"/>
@@ -1664,7 +1664,7 @@
       <c r="L41" s="8"/>
       <c r="M41" s="5"/>
     </row>
-    <row r="42" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="12"/>
       <c r="B42" s="4"/>
       <c r="C42" s="7"/>
@@ -1679,7 +1679,7 @@
       <c r="L42" s="7"/>
       <c r="M42" s="5"/>
     </row>
-    <row r="43" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="12"/>
       <c r="B43" s="4"/>
       <c r="C43" s="8"/>
@@ -1694,7 +1694,7 @@
       <c r="L43" s="8"/>
       <c r="M43" s="5"/>
     </row>
-    <row r="44" spans="1:13" ht="28.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="12"/>
       <c r="B44" s="4"/>
       <c r="C44" s="7"/>
@@ -1709,7 +1709,7 @@
       <c r="L44" s="7"/>
       <c r="M44" s="5"/>
     </row>
-    <row r="45" spans="1:13" ht="6.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:13" ht="6.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="12"/>
       <c r="B45" s="4"/>
       <c r="C45" s="8"/>
@@ -1724,7 +1724,7 @@
       <c r="L45" s="8"/>
       <c r="M45" s="5"/>
     </row>
-    <row r="46" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="12"/>
       <c r="B46" s="4"/>
       <c r="C46" s="7"/>
@@ -1739,7 +1739,7 @@
       <c r="L46" s="7"/>
       <c r="M46" s="5"/>
     </row>
-    <row r="47" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="12"/>
       <c r="B47" s="4"/>
       <c r="C47" s="8"/>
@@ -1754,7 +1754,7 @@
       <c r="L47" s="8"/>
       <c r="M47" s="5"/>
     </row>
-    <row r="48" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="12"/>
       <c r="B48" s="4"/>
       <c r="C48" s="7"/>
@@ -1769,7 +1769,7 @@
       <c r="L48" s="7"/>
       <c r="M48" s="5"/>
     </row>
-    <row r="49" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="12"/>
       <c r="B49" s="4"/>
       <c r="C49" s="8"/>
@@ -1784,7 +1784,7 @@
       <c r="L49" s="8"/>
       <c r="M49" s="5"/>
     </row>
-    <row r="50" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="12"/>
       <c r="B50" s="4"/>
       <c r="C50" s="7"/>
@@ -1799,7 +1799,7 @@
       <c r="L50" s="7"/>
       <c r="M50" s="5"/>
     </row>
-    <row r="51" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="12"/>
       <c r="B51" s="4"/>
       <c r="C51" s="8"/>
@@ -1814,7 +1814,7 @@
       <c r="L51" s="8"/>
       <c r="M51" s="5"/>
     </row>
-    <row r="52" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="12"/>
       <c r="B52" s="4"/>
       <c r="C52" s="7"/>
@@ -1829,7 +1829,7 @@
       <c r="L52" s="7"/>
       <c r="M52" s="5"/>
     </row>
-    <row r="53" spans="1:13" ht="28.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:13" ht="28.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="12"/>
       <c r="B53" s="4"/>
       <c r="C53" s="8"/>
@@ -1844,7 +1844,7 @@
       <c r="L53" s="8"/>
       <c r="M53" s="5"/>
     </row>
-    <row r="54" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="12"/>
       <c r="B54" s="4"/>
       <c r="C54" s="7"/>
@@ -1859,7 +1859,7 @@
       <c r="L54" s="7"/>
       <c r="M54" s="5"/>
     </row>
-    <row r="55" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12"/>
       <c r="B55" s="4"/>
       <c r="C55" s="8"/>
@@ -1874,7 +1874,7 @@
       <c r="L55" s="8"/>
       <c r="M55" s="5"/>
     </row>
-    <row r="56" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="12"/>
       <c r="B56" s="4"/>
       <c r="C56" s="7"/>
@@ -1889,7 +1889,7 @@
       <c r="L56" s="7"/>
       <c r="M56" s="5"/>
     </row>
-    <row r="57" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12"/>
       <c r="B57" s="4"/>
       <c r="C57" s="8"/>
@@ -1904,7 +1904,7 @@
       <c r="L57" s="8"/>
       <c r="M57" s="5"/>
     </row>
-    <row r="58" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="12"/>
       <c r="B58" s="4"/>
       <c r="C58" s="7"/>
@@ -1919,7 +1919,7 @@
       <c r="L58" s="7"/>
       <c r="M58" s="5"/>
     </row>
-    <row r="59" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="12"/>
       <c r="B59" s="4"/>
       <c r="C59" s="8"/>
@@ -1934,7 +1934,7 @@
       <c r="L59" s="8"/>
       <c r="M59" s="5"/>
     </row>
-    <row r="60" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="12"/>
       <c r="B60" s="4"/>
       <c r="C60" s="7"/>
@@ -1949,7 +1949,7 @@
       <c r="L60" s="7"/>
       <c r="M60" s="5"/>
     </row>
-    <row r="61" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="12"/>
       <c r="B61" s="4"/>
       <c r="C61" s="8"/>
@@ -1964,7 +1964,7 @@
       <c r="L61" s="8"/>
       <c r="M61" s="5"/>
     </row>
-    <row r="62" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="12"/>
       <c r="B62" s="4"/>
       <c r="C62" s="7"/>
@@ -1979,7 +1979,7 @@
       <c r="L62" s="7"/>
       <c r="M62" s="5"/>
     </row>
-    <row r="63" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="12"/>
       <c r="B63" s="10"/>
       <c r="C63" s="8"/>
@@ -1994,7 +1994,7 @@
       <c r="L63" s="8"/>
       <c r="M63" s="11"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="12"/>
       <c r="B64" s="1"/>
       <c r="C64" s="12"/>
@@ -2002,52 +2002,52 @@
       <c r="E64" s="12"/>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
-      <c r="H64" s="54" t="s">
-        <v>35</v>
-      </c>
-      <c r="I64" s="54"/>
-      <c r="J64" s="54"/>
-      <c r="K64" s="54"/>
-      <c r="L64" s="54"/>
-      <c r="M64" s="25"/>
-    </row>
-    <row r="65" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H64" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="I64" s="33"/>
+      <c r="J64" s="33"/>
+      <c r="K64" s="33"/>
+      <c r="L64" s="33"/>
+      <c r="M64" s="34"/>
+    </row>
+    <row r="65" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="12"/>
       <c r="B65" s="4"/>
-      <c r="C65" s="55" t="s">
-        <v>31</v>
-      </c>
-      <c r="D65" s="55"/>
-      <c r="E65" s="55"/>
-      <c r="F65" s="55"/>
+      <c r="C65" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D65" s="35"/>
+      <c r="E65" s="35"/>
+      <c r="F65" s="35"/>
       <c r="G65" s="12"/>
-      <c r="H65" s="55"/>
-      <c r="I65" s="55"/>
-      <c r="J65" s="55"/>
-      <c r="K65" s="55"/>
-      <c r="L65" s="55"/>
-      <c r="M65" s="56"/>
-    </row>
-    <row r="66" spans="1:13" ht="16" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="H65" s="35"/>
+      <c r="I65" s="35"/>
+      <c r="J65" s="35"/>
+      <c r="K65" s="35"/>
+      <c r="L65" s="35"/>
+      <c r="M65" s="36"/>
+    </row>
+    <row r="66" spans="1:13" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A66" s="12"/>
       <c r="B66" s="4"/>
-      <c r="C66" s="45" t="s">
+      <c r="C66" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="D66" s="45"/>
-      <c r="E66" s="45"/>
-      <c r="F66" s="45"/>
+      <c r="D66" s="23"/>
+      <c r="E66" s="23"/>
+      <c r="F66" s="23"/>
       <c r="G66" s="12"/>
-      <c r="H66" s="45" t="s">
+      <c r="H66" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="I66" s="45"/>
-      <c r="J66" s="45"/>
-      <c r="K66" s="45"/>
-      <c r="L66" s="45"/>
-      <c r="M66" s="46"/>
-    </row>
-    <row r="67" spans="1:13" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="I66" s="23"/>
+      <c r="J66" s="23"/>
+      <c r="K66" s="23"/>
+      <c r="L66" s="23"/>
+      <c r="M66" s="24"/>
+    </row>
+    <row r="67" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A67" s="12"/>
       <c r="B67" s="4"/>
       <c r="C67" s="18"/>
@@ -2062,7 +2062,7 @@
       <c r="L67" s="12"/>
       <c r="M67" s="19"/>
     </row>
-    <row r="68" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="12"/>
       <c r="B68" s="4"/>
       <c r="D68" s="7"/>
@@ -2076,7 +2076,7 @@
       <c r="L68" s="7"/>
       <c r="M68" s="5"/>
     </row>
-    <row r="69" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="12"/>
       <c r="B69" s="10"/>
       <c r="C69" s="8"/>
@@ -2093,6 +2093,16 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="E6:L6"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="E9:L9"/>
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="B2:C4"/>
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="D3:I4"/>
     <mergeCell ref="C66:F66"/>
     <mergeCell ref="H66:M66"/>
     <mergeCell ref="F11:L11"/>
@@ -2109,16 +2119,6 @@
     <mergeCell ref="I19:L19"/>
     <mergeCell ref="H64:M65"/>
     <mergeCell ref="C65:F65"/>
-    <mergeCell ref="E6:L6"/>
-    <mergeCell ref="E8:L8"/>
-    <mergeCell ref="E9:L9"/>
-    <mergeCell ref="E20:L20"/>
-    <mergeCell ref="B2:C4"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="D3:I4"/>
   </mergeCells>
   <pageMargins left="0.9055118110236221" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.51181102362204722"/>
   <pageSetup paperSize="5" scale="72" orientation="portrait" r:id="rId1"/>

</xml_diff>